<commit_message>
downloaded a chapter of social epist, lrc attendance and essay grades
</commit_message>
<xml_diff>
--- a/lrc_attnd_for_R.xlsx
+++ b/lrc_attnd_for_R.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kom11/Documents/GitHub/phd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB46B5C-BF42-9F4F-9E7A-DAC5CDA6C714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10B3B8A-C766-EC4C-9EC8-7E4C0D60740E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8920" yWindow="-20920" windowWidth="16340" windowHeight="19280" xr2:uid="{B94DB17C-919E-1C4A-B529-5E14F6099E2A}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="11340" windowHeight="19780" xr2:uid="{B94DB17C-919E-1C4A-B529-5E14F6099E2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Essay 2" sheetId="2" r:id="rId2"/>
+    <sheet name="essay 3" sheetId="3" r:id="rId2"/>
+    <sheet name="Essay 2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="122">
   <si>
     <t>Avery</t>
   </si>
@@ -349,13 +350,67 @@
   </si>
   <si>
     <t>B+</t>
+  </si>
+  <si>
+    <t>berry</t>
+  </si>
+  <si>
+    <t>hazony</t>
+  </si>
+  <si>
+    <t>oak</t>
+  </si>
+  <si>
+    <t>burke</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>deneen</t>
+  </si>
+  <si>
+    <t>deen</t>
+  </si>
+  <si>
+    <t>lowry</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>93/94</t>
+  </si>
+  <si>
+    <t>92/90</t>
+  </si>
+  <si>
+    <t>for AM</t>
+  </si>
+  <si>
+    <t>AM</t>
+  </si>
+  <si>
+    <t>85???</t>
+  </si>
+  <si>
+    <t>XXX</t>
+  </si>
+  <si>
+    <t>87-90</t>
+  </si>
+  <si>
+    <t>91 or 93</t>
+  </si>
+  <si>
+    <t>in class</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -382,6 +437,20 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -412,7 +481,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -420,6 +489,8 @@
     <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="16" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,10 +507,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -763,8 +830,12 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="3" max="20" width="10.83203125" customWidth="1"/>
-    <col min="21" max="24" width="23.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="20" width="10.83203125" hidden="1" customWidth="1"/>
+    <col min="21" max="24" width="23.83203125" hidden="1" customWidth="1"/>
+    <col min="25" max="31" width="0" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="7.1640625" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -909,7 +980,7 @@
         <v>1</v>
       </c>
       <c r="U2" s="1">
-        <f>SUM(C2:T2)</f>
+        <f t="shared" ref="U2:U40" si="0">SUM(C2:T2)</f>
         <v>15</v>
       </c>
       <c r="V2" s="6">
@@ -923,6 +994,9 @@
       <c r="X2" s="6" t="s">
         <v>98</v>
       </c>
+      <c r="AG2">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -953,19 +1027,22 @@
         <v>2</v>
       </c>
       <c r="U3" s="1">
-        <f>SUM(C3:T3)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="V3" s="6">
-        <f t="shared" ref="V3:V39" si="0">U3/36</f>
+        <f t="shared" ref="V3:V39" si="1">U3/36</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="W3" s="6">
-        <f t="shared" ref="W3:W39" si="1" xml:space="preserve"> U3/22</f>
+        <f t="shared" ref="W3:W39" si="2" xml:space="preserve"> U3/22</f>
         <v>0.54545454545454541</v>
       </c>
       <c r="X3" s="6" t="s">
         <v>99</v>
+      </c>
+      <c r="AG3">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.2">
@@ -988,15 +1065,15 @@
         <v>2</v>
       </c>
       <c r="U4" s="1">
-        <f>SUM(C4:T4)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="V4" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="W4" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.36363636363636365</v>
       </c>
       <c r="X4" s="6" t="s">
@@ -1044,15 +1121,15 @@
         <v>2</v>
       </c>
       <c r="U5" s="1">
-        <f>SUM(C5:T5)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="V5" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="W5" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.90909090909090906</v>
       </c>
       <c r="X5" s="6" t="s">
@@ -1094,19 +1171,22 @@
         <v>2</v>
       </c>
       <c r="U6" s="1">
-        <f>SUM(C6:T6)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="V6" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.47222222222222221</v>
       </c>
       <c r="W6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77272727272727271</v>
       </c>
       <c r="X6" s="6" t="s">
         <v>102</v>
+      </c>
+      <c r="AG6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
@@ -1120,15 +1200,15 @@
         <v>2</v>
       </c>
       <c r="U7" s="1">
-        <f>SUM(C7:T7)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="V7" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="W7" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.0909090909090912E-2</v>
       </c>
       <c r="X7" s="6" t="s">
@@ -1149,15 +1229,15 @@
         <v>1</v>
       </c>
       <c r="U8" s="1">
-        <f>SUM(C8:T8)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="V8" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="W8" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.13636363636363635</v>
       </c>
       <c r="X8" s="6" t="s">
@@ -1193,19 +1273,22 @@
         <v>2</v>
       </c>
       <c r="U9" s="1">
-        <f>SUM(C9:T9)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="V9" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.3888888888888889</v>
       </c>
       <c r="W9" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.63636363636363635</v>
       </c>
       <c r="X9" s="6" t="s">
         <v>99</v>
+      </c>
+      <c r="AG9">
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.2">
@@ -1225,19 +1308,22 @@
         <v>2</v>
       </c>
       <c r="U10" s="1">
-        <f>SUM(C10:T10)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="V10" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.16666666666666666</v>
       </c>
       <c r="W10" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.27272727272727271</v>
       </c>
       <c r="X10" s="6" t="s">
         <v>100</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:36" x14ac:dyDescent="0.2">
@@ -1275,19 +1361,22 @@
         <v>2</v>
       </c>
       <c r="U11" s="1">
-        <f>SUM(C11:T11)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="V11" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.47222222222222221</v>
       </c>
       <c r="W11" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77272727272727271</v>
       </c>
       <c r="X11" s="6" t="s">
         <v>102</v>
+      </c>
+      <c r="AG11">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:36" x14ac:dyDescent="0.2">
@@ -1328,19 +1417,22 @@
         <v>2</v>
       </c>
       <c r="U12" s="1">
-        <f>SUM(C12:T12)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="V12" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="W12" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.90909090909090906</v>
       </c>
       <c r="X12" s="6" t="s">
         <v>101</v>
+      </c>
+      <c r="AG12">
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.2">
@@ -1378,15 +1470,15 @@
         <v>2</v>
       </c>
       <c r="U13" s="1">
-        <f>SUM(C13:T13)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="V13" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.47222222222222221</v>
       </c>
       <c r="W13" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77272727272727271</v>
       </c>
       <c r="X13" s="6" t="s">
@@ -1416,19 +1508,22 @@
         <v>2</v>
       </c>
       <c r="U14" s="1">
-        <f>SUM(C14:T14)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="V14" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.27777777777777779</v>
       </c>
       <c r="W14" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.45454545454545453</v>
       </c>
       <c r="X14" s="6" t="s">
         <v>100</v>
+      </c>
+      <c r="AG14">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.2">
@@ -1466,15 +1561,15 @@
         <v>2</v>
       </c>
       <c r="U15" s="1">
-        <f>SUM(C15:T15)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="V15" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="W15" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.81818181818181823</v>
       </c>
       <c r="X15" s="6" t="s">
@@ -1507,20 +1602,23 @@
         <v>2</v>
       </c>
       <c r="U16" s="1">
-        <f>SUM(C16:T16)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="V16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.30555555555555558</v>
       </c>
       <c r="W16" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="X16" s="6"/>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1549,20 +1647,23 @@
         <v>2</v>
       </c>
       <c r="U17" s="1">
-        <f>SUM(C17:T17)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="V17" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.3611111111111111</v>
       </c>
       <c r="W17" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.59090909090909094</v>
       </c>
       <c r="X17" s="6"/>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1603,20 +1704,23 @@
         <v>2</v>
       </c>
       <c r="U18" s="1">
-        <f>SUM(C18:T18)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="V18" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.61111111111111116</v>
       </c>
       <c r="W18" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="X18" s="6"/>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1642,20 +1746,23 @@
         <v>2</v>
       </c>
       <c r="U19" s="1">
-        <f>SUM(C19:T19)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="V19" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="W19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.54545454545454541</v>
       </c>
       <c r="X19" s="6"/>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1678,20 +1785,23 @@
         <v>2</v>
       </c>
       <c r="U20" s="1">
-        <f>SUM(C20:T20)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="V20" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.27777777777777779</v>
       </c>
       <c r="W20" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.45454545454545453</v>
       </c>
       <c r="X20" s="6"/>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1714,20 +1824,23 @@
         <v>2</v>
       </c>
       <c r="U21" s="1">
-        <f>SUM(C21:T21)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="V21" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
       <c r="W21" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.40909090909090912</v>
       </c>
       <c r="X21" s="6"/>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG21" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1765,20 +1878,20 @@
         <v>2</v>
       </c>
       <c r="U22" s="1">
-        <f>SUM(C22:T22)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="V22" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.3611111111111111</v>
       </c>
       <c r="W22" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.59090909090909094</v>
       </c>
       <c r="X22" s="6"/>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1789,20 +1902,20 @@
         <v>2</v>
       </c>
       <c r="U23" s="1">
-        <f>SUM(C23:T23)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="V23" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="W23" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.0909090909090912E-2</v>
       </c>
       <c r="X23" s="6"/>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1813,20 +1926,20 @@
         <v>2</v>
       </c>
       <c r="U24" s="1">
-        <f>SUM(C24:T24)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="V24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="W24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.0909090909090912E-2</v>
       </c>
       <c r="X24" s="6"/>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -1840,20 +1953,23 @@
         <v>2</v>
       </c>
       <c r="U25" s="1">
-        <f>SUM(C25:T25)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="V25" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1111111111111111</v>
       </c>
       <c r="W25" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.18181818181818182</v>
       </c>
       <c r="X25" s="6"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1888,20 +2004,23 @@
         <v>2</v>
       </c>
       <c r="U26" s="1">
-        <f>SUM(C26:T26)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="V26" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.47222222222222221</v>
       </c>
       <c r="W26" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77272727272727271</v>
       </c>
       <c r="X26" s="6"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -1927,20 +2046,23 @@
         <v>2</v>
       </c>
       <c r="U27" s="1">
-        <f>SUM(C27:T27)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="V27" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="W27" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.54545454545454541</v>
       </c>
       <c r="X27" s="6"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>52</v>
       </c>
@@ -1951,20 +2073,23 @@
         <v>2</v>
       </c>
       <c r="U28" s="1">
-        <f>SUM(C28:T28)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="V28" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5555555555555552E-2</v>
       </c>
       <c r="W28" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.0909090909090912E-2</v>
       </c>
       <c r="X28" s="6"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -1993,20 +2118,23 @@
         <v>2</v>
       </c>
       <c r="U29" s="1">
-        <f>SUM(C29:T29)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="V29" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.3888888888888889</v>
       </c>
       <c r="W29" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.63636363636363635</v>
       </c>
       <c r="X29" s="6"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>54</v>
       </c>
@@ -2029,20 +2157,23 @@
         <v>2</v>
       </c>
       <c r="U30" s="1">
-        <f>SUM(C30:T30)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="V30" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.27777777777777779</v>
       </c>
       <c r="W30" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.45454545454545453</v>
       </c>
       <c r="X30" s="6"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>56</v>
       </c>
@@ -2065,20 +2196,23 @@
         <v>2</v>
       </c>
       <c r="U31" s="1">
-        <f>SUM(C31:T31)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="V31" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.27777777777777779</v>
       </c>
       <c r="W31" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.45454545454545453</v>
       </c>
       <c r="X31" s="6"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>58</v>
       </c>
@@ -2095,20 +2229,23 @@
         <v>2</v>
       </c>
       <c r="U32" s="1">
-        <f>SUM(C32:T32)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="V32" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1111111111111111</v>
       </c>
       <c r="W32" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.18181818181818182</v>
       </c>
       <c r="X32" s="6"/>
-    </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>60</v>
       </c>
@@ -2155,20 +2292,23 @@
         <v>2</v>
       </c>
       <c r="U33" s="1">
-        <f>SUM(C33:T33)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="V33" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.61111111111111116</v>
       </c>
       <c r="W33" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="X33" s="6"/>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>62</v>
       </c>
@@ -2209,20 +2349,23 @@
         <v>2</v>
       </c>
       <c r="U34" s="1">
-        <f>SUM(C34:T34)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="V34" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.58333333333333337</v>
       </c>
       <c r="W34" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.95454545454545459</v>
       </c>
       <c r="X34" s="6"/>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>64</v>
       </c>
@@ -2260,20 +2403,23 @@
         <v>2</v>
       </c>
       <c r="U35" s="1">
-        <f>SUM(C35:T35)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="V35" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.52777777777777779</v>
       </c>
       <c r="W35" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.86363636363636365</v>
       </c>
       <c r="X35" s="6"/>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>66</v>
       </c>
@@ -2293,20 +2439,20 @@
         <v>2</v>
       </c>
       <c r="U36" s="1">
-        <f>SUM(C36:T36)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="V36" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.19444444444444445</v>
       </c>
       <c r="W36" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.31818181818181818</v>
       </c>
       <c r="X36" s="6"/>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -2314,20 +2460,20 @@
         <v>69</v>
       </c>
       <c r="U37" s="1">
-        <f>SUM(C37:T37)</f>
-        <v>0</v>
-      </c>
-      <c r="V37" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="W37" s="6">
+      <c r="V37" s="6">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="W37" s="6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="X37" s="6"/>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>70</v>
       </c>
@@ -2350,20 +2496,23 @@
         <v>2</v>
       </c>
       <c r="U38" s="1">
-        <f>SUM(C38:T38)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="V38" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
       <c r="W38" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.40909090909090912</v>
       </c>
       <c r="X38" s="6"/>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>72</v>
       </c>
@@ -2389,20 +2538,23 @@
         <v>2</v>
       </c>
       <c r="U39" s="1">
-        <f>SUM(C39:T39)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="V39" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.27777777777777779</v>
       </c>
       <c r="W39" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.45454545454545453</v>
       </c>
       <c r="X39" s="6"/>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="AG39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>95</v>
       </c>
@@ -2464,7 +2616,7 @@
         <v>2</v>
       </c>
       <c r="U40" s="1">
-        <f>SUM(C40:T40)</f>
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
     </row>
@@ -2474,6 +2626,742 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ECBB356-6AF7-8740-A0ED-9A14B24F1E9D}">
+  <dimension ref="A1:I40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2">
+        <v>97</v>
+      </c>
+      <c r="E2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3">
+        <v>94</v>
+      </c>
+      <c r="E3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E5" t="s">
+        <v>107</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6">
+        <v>96</v>
+      </c>
+      <c r="E6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7">
+        <v>93</v>
+      </c>
+      <c r="E7" t="s">
+        <v>112</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8">
+        <v>93</v>
+      </c>
+      <c r="E8" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9">
+        <v>93</v>
+      </c>
+      <c r="E9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" t="s">
+        <v>110</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11">
+        <v>95</v>
+      </c>
+      <c r="E11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13">
+        <v>92</v>
+      </c>
+      <c r="E13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>111</v>
+      </c>
+      <c r="D15">
+        <v>96</v>
+      </c>
+      <c r="E15" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16">
+        <v>97</v>
+      </c>
+      <c r="E16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" t="s">
+        <v>116</v>
+      </c>
+      <c r="E18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19">
+        <v>98</v>
+      </c>
+      <c r="E19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" t="s">
+        <v>116</v>
+      </c>
+      <c r="E22" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" t="s">
+        <v>119</v>
+      </c>
+      <c r="E23" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" t="s">
+        <v>113</v>
+      </c>
+      <c r="E24" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25">
+        <v>90</v>
+      </c>
+      <c r="E25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" t="s">
+        <v>114</v>
+      </c>
+      <c r="E26" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" t="s">
+        <v>117</v>
+      </c>
+      <c r="E27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" t="s">
+        <v>105</v>
+      </c>
+      <c r="D28" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" t="s">
+        <v>105</v>
+      </c>
+      <c r="D29">
+        <v>98</v>
+      </c>
+      <c r="E29" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D30">
+        <v>95</v>
+      </c>
+      <c r="E30" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" t="s">
+        <v>109</v>
+      </c>
+      <c r="D31">
+        <v>97</v>
+      </c>
+      <c r="E31" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" t="s">
+        <v>105</v>
+      </c>
+      <c r="D32">
+        <v>92</v>
+      </c>
+      <c r="E32" t="s">
+        <v>111</v>
+      </c>
+      <c r="F32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" t="s">
+        <v>120</v>
+      </c>
+      <c r="E33" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34">
+        <v>95</v>
+      </c>
+      <c r="E34" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35">
+        <v>98</v>
+      </c>
+      <c r="E35" t="s">
+        <v>106</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E36" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" t="s">
+        <v>110</v>
+      </c>
+      <c r="D37" t="s">
+        <v>118</v>
+      </c>
+      <c r="E37" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" t="s">
+        <v>109</v>
+      </c>
+      <c r="D39" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D40">
+    <sortCondition ref="B2:B40"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C73BCEF-4552-CE4D-BE68-23600D60C9E9}">
   <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
doing end of semester attendance
</commit_message>
<xml_diff>
--- a/lrc_attnd_for_R.xlsx
+++ b/lrc_attnd_for_R.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kom11/Documents/GitHub/phd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FEC267-7D7A-1C4E-8FAD-143CEFDDB3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2D8B85-1BFF-4D46-A289-6C4AA2898716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="10000" windowHeight="19780" xr2:uid="{B94DB17C-919E-1C4A-B529-5E14F6099E2A}"/>
+    <workbookView xWindow="12760" yWindow="680" windowWidth="19640" windowHeight="19780" xr2:uid="{B94DB17C-919E-1C4A-B529-5E14F6099E2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="121">
   <si>
     <t>Avery</t>
   </si>
@@ -401,12 +401,6 @@
   </si>
   <si>
     <t>91 or 93</t>
-  </si>
-  <si>
-    <t>in class</t>
-  </si>
-  <si>
-    <t>?</t>
   </si>
 </sst>
 </file>
@@ -484,7 +478,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -494,8 +488,6 @@
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -836,12 +828,11 @@
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" customWidth="1"/>
-    <col min="3" max="20" width="10.83203125" hidden="1" customWidth="1"/>
-    <col min="21" max="24" width="23.83203125" hidden="1" customWidth="1"/>
-    <col min="25" max="31" width="0" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="7.1640625" hidden="1" customWidth="1"/>
+    <col min="3" max="20" width="10.83203125" customWidth="1"/>
+    <col min="21" max="24" width="23.83203125" customWidth="1"/>
+    <col min="25" max="31" width="10.83203125" customWidth="1"/>
+    <col min="32" max="32" width="7.1640625" customWidth="1"/>
     <col min="33" max="33" width="15.5" customWidth="1"/>
-    <col min="35" max="35" width="10.83203125" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -932,27 +923,19 @@
       <c r="AC1" s="4">
         <v>46114</v>
       </c>
-      <c r="AD1" s="4">
-        <v>46117</v>
-      </c>
-      <c r="AE1" s="4">
-        <v>46119</v>
-      </c>
-      <c r="AF1" s="4">
-        <v>46121</v>
-      </c>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
       <c r="AG1" s="4">
         <v>46126</v>
       </c>
       <c r="AH1" s="4">
         <v>46128</v>
       </c>
-      <c r="AI1" s="9">
+      <c r="AI1" s="4">
         <v>46133</v>
       </c>
-      <c r="AJ1" s="4">
-        <v>46142</v>
-      </c>
+      <c r="AJ1" s="4"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1006,7 +989,7 @@
       <c r="AH2">
         <v>2</v>
       </c>
-      <c r="AI2" s="10">
+      <c r="AI2">
         <v>1</v>
       </c>
     </row>
@@ -1059,7 +1042,7 @@
       <c r="AH3">
         <v>2</v>
       </c>
-      <c r="AI3" s="10">
+      <c r="AI3">
         <v>1</v>
       </c>
     </row>
@@ -1097,7 +1080,7 @@
       <c r="X4" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="AI4" s="10">
+      <c r="AI4">
         <v>2</v>
       </c>
     </row>
@@ -1212,7 +1195,7 @@
       <c r="AG6">
         <v>2</v>
       </c>
-      <c r="AI6" s="10">
+      <c r="AI6">
         <v>2</v>
       </c>
     </row>
@@ -1241,8 +1224,8 @@
       <c r="X7" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="AH7" t="s">
-        <v>122</v>
+      <c r="AH7">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.2">
@@ -1318,9 +1301,9 @@
         <v>99</v>
       </c>
       <c r="AG9">
-        <v>10</v>
-      </c>
-      <c r="AI9" s="10">
+        <v>2</v>
+      </c>
+      <c r="AI9">
         <v>2</v>
       </c>
     </row>
@@ -1355,10 +1338,10 @@
       <c r="X10" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="AG10" t="s">
-        <v>121</v>
-      </c>
-      <c r="AI10" s="10">
+      <c r="AG10">
+        <v>1</v>
+      </c>
+      <c r="AI10">
         <v>2</v>
       </c>
     </row>
@@ -1473,7 +1456,7 @@
       <c r="AG12">
         <v>2</v>
       </c>
-      <c r="AI12" s="10">
+      <c r="AI12">
         <v>2</v>
       </c>
     </row>
@@ -1526,7 +1509,7 @@
       <c r="X13" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="AI13" s="10">
+      <c r="AI13">
         <v>2</v>
       </c>
     </row>
@@ -1626,7 +1609,7 @@
       <c r="AH15">
         <v>2</v>
       </c>
-      <c r="AI15" s="10">
+      <c r="AI15">
         <v>2</v>
       </c>
     </row>
@@ -1674,7 +1657,7 @@
       <c r="AH16">
         <v>2</v>
       </c>
-      <c r="AI16" s="10">
+      <c r="AI16">
         <v>2</v>
       </c>
     </row>
@@ -1785,7 +1768,7 @@
       <c r="AH18">
         <v>2</v>
       </c>
-      <c r="AI18" s="10">
+      <c r="AI18">
         <v>2</v>
       </c>
     </row>
@@ -1833,7 +1816,7 @@
       <c r="AH19">
         <v>2</v>
       </c>
-      <c r="AI19" s="10">
+      <c r="AI19">
         <v>2</v>
       </c>
     </row>
@@ -1878,7 +1861,7 @@
       <c r="AH20">
         <v>2</v>
       </c>
-      <c r="AI20" s="10">
+      <c r="AI20">
         <v>2</v>
       </c>
     </row>
@@ -1923,7 +1906,7 @@
       <c r="AH21">
         <v>2</v>
       </c>
-      <c r="AI21" s="10">
+      <c r="AI21">
         <v>2</v>
       </c>
     </row>
@@ -2031,7 +2014,7 @@
       <c r="AH24">
         <v>2</v>
       </c>
-      <c r="AI24" s="10">
+      <c r="AI24">
         <v>2</v>
       </c>
     </row>
@@ -2118,7 +2101,7 @@
       <c r="AH26">
         <v>2</v>
       </c>
-      <c r="AI26" s="10">
+      <c r="AI26">
         <v>2</v>
       </c>
     </row>
@@ -2166,7 +2149,7 @@
       <c r="AH27">
         <v>2</v>
       </c>
-      <c r="AI27" s="10">
+      <c r="AI27">
         <v>2</v>
       </c>
     </row>
@@ -2199,7 +2182,7 @@
       <c r="AH28">
         <v>2</v>
       </c>
-      <c r="AI28" s="10">
+      <c r="AI28">
         <v>2</v>
       </c>
     </row>
@@ -2247,7 +2230,7 @@
       <c r="AG29">
         <v>2</v>
       </c>
-      <c r="AI29" s="10">
+      <c r="AI29">
         <v>1</v>
       </c>
     </row>
@@ -2367,8 +2350,8 @@
       <c r="AG32">
         <v>2</v>
       </c>
-      <c r="AH32" t="s">
-        <v>122</v>
+      <c r="AH32">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:35" x14ac:dyDescent="0.2">
@@ -2550,7 +2533,7 @@
       <c r="AG35">
         <v>2</v>
       </c>
-      <c r="AI35" s="10">
+      <c r="AI35">
         <v>2</v>
       </c>
     </row>
@@ -2589,7 +2572,7 @@
       <c r="AH36">
         <v>2</v>
       </c>
-      <c r="AI36" s="10">
+      <c r="AI36">
         <v>2</v>
       </c>
     </row>
@@ -2700,7 +2683,7 @@
       <c r="AH39">
         <v>2</v>
       </c>
-      <c r="AI39" s="10">
+      <c r="AI39">
         <v>2</v>
       </c>
     </row>

</xml_diff>